<commit_message>
feat: settle name-priority logic and refresh 3-year simulation scenarios (April 11)
</commit_message>
<xml_diff>
--- a/exports/monthly_ledger_excel/DEATH_VALLEY/ledger_2026-05.xlsx
+++ b/exports/monthly_ledger_excel/DEATH_VALLEY/ledger_2026-05.xlsx
@@ -397,44 +397,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>id</v>
+        <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>date</v>
+        <v>날짜</v>
       </c>
       <c r="C1" t="str">
-        <v>description</v>
+        <v>적요</v>
       </c>
       <c r="D1" t="str">
-        <v>vendor</v>
+        <v>거래처</v>
       </c>
       <c r="E1" t="str">
-        <v>debitAccount</v>
+        <v>차변계정</v>
       </c>
       <c r="F1" t="str">
-        <v>debitAccountId</v>
+        <v>차변ID</v>
       </c>
       <c r="G1" t="str">
-        <v>creditAccount</v>
+        <v>대변계정</v>
       </c>
       <c r="H1" t="str">
-        <v>creditAccountId</v>
+        <v>대변ID</v>
       </c>
       <c r="I1" t="str">
-        <v>amount</v>
+        <v>금액</v>
       </c>
       <c r="J1" t="str">
-        <v>vat</v>
+        <v>부가세</v>
       </c>
       <c r="K1" t="str">
-        <v>type</v>
+        <v>유형</v>
       </c>
       <c r="L1" t="str">
-        <v>status</v>
+        <v>상태</v>
       </c>
     </row>
     <row r="2">
@@ -515,22 +515,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>RENT-2026-5</v>
+        <v>OH-2026-5</v>
       </c>
       <c r="B4" t="str">
         <v>2026-05-28</v>
       </c>
       <c r="C4" t="str">
-        <v>[RENT] 공간 임차료</v>
+        <v>[EXP] 인건비 부대비용</v>
       </c>
       <c r="D4" t="str">
-        <v>Bldg</v>
+        <v>Staff Overhead</v>
       </c>
       <c r="E4" t="str">
-        <v>임차료</v>
+        <v>세금과공과</v>
       </c>
       <c r="F4" t="str">
-        <v>acc_819</v>
+        <v>acc_817</v>
       </c>
       <c r="G4" t="str">
         <v>보통예금</v>
@@ -539,10 +539,10 @@
         <v>acc_103</v>
       </c>
       <c r="I4">
-        <v>5000000</v>
+        <v>2745000</v>
       </c>
       <c r="J4">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="K4" t="str">
         <v>Expense</v>
@@ -553,45 +553,159 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MKT-2026-5</v>
+        <v>RENT-AP-2026-5</v>
       </c>
       <c r="B5" t="str">
         <v>2026-05-28</v>
       </c>
       <c r="C5" t="str">
-        <v>[MKT] 마케팅비</v>
+        <v>[RENT] 공간 임차료 청구</v>
       </c>
       <c r="D5" t="str">
-        <v>Google</v>
+        <v>Bldg</v>
       </c>
       <c r="E5" t="str">
-        <v>마케팅비</v>
+        <v>임차료</v>
       </c>
       <c r="F5" t="str">
-        <v>acc_830</v>
+        <v>acc_816</v>
       </c>
       <c r="G5" t="str">
-        <v>보통예금</v>
+        <v>미지급금</v>
       </c>
       <c r="H5" t="str">
-        <v>acc_103</v>
+        <v>acc_253</v>
       </c>
       <c r="I5">
-        <v>3000000</v>
+        <v>5000000</v>
       </c>
       <c r="J5">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="K5" t="str">
         <v>Expense</v>
       </c>
       <c r="L5" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>RENT-PAY-2026-5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="C6" t="str">
+        <v>[SETTLE] 임차료 결제 (90%)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Bldg</v>
+      </c>
+      <c r="E6" t="str">
+        <v>미지급금</v>
+      </c>
+      <c r="F6" t="str">
+        <v>acc_253</v>
+      </c>
+      <c r="G6" t="str">
+        <v>보통예금</v>
+      </c>
+      <c r="H6" t="str">
+        <v>acc_103</v>
+      </c>
+      <c r="I6">
+        <v>4950000</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>MKT-AP-2026-5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="C7" t="str">
+        <v>[MKT] 마케팅비 청구</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Google/FB</v>
+      </c>
+      <c r="E7" t="str">
+        <v>광고선전비</v>
+      </c>
+      <c r="F7" t="str">
+        <v>acc_826</v>
+      </c>
+      <c r="G7" t="str">
+        <v>미지급금</v>
+      </c>
+      <c r="H7" t="str">
+        <v>acc_253</v>
+      </c>
+      <c r="I7">
+        <v>4000000</v>
+      </c>
+      <c r="J7">
+        <v>400000</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>MKT-PAY-2026-5</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="C8" t="str">
+        <v>[SETTLE] 마케팅비 결제 (80% 우선집행)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Google/FB</v>
+      </c>
+      <c r="E8" t="str">
+        <v>미지급금</v>
+      </c>
+      <c r="F8" t="str">
+        <v>acc_253</v>
+      </c>
+      <c r="G8" t="str">
+        <v>보통예금</v>
+      </c>
+      <c r="H8" t="str">
+        <v>acc_103</v>
+      </c>
+      <c r="I8">
+        <v>3520000</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="L8" t="str">
         <v>Approved</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CHORE: Accounting Engine Integrity Restored (End-to-End Verified)
</commit_message>
<xml_diff>
--- a/exports/monthly_ledger_excel/DEATH_VALLEY/ledger_2026-05.xlsx
+++ b/exports/monthly_ledger_excel/DEATH_VALLEY/ledger_2026-05.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,7 +483,7 @@
         <v>2026-05-28</v>
       </c>
       <c r="C3" t="str">
-        <v>[PAY] 정기 인건비</v>
+        <v>[PAY] 당월 급여 지급</v>
       </c>
       <c r="D3" t="str">
         <v>Staff</v>
@@ -521,7 +521,7 @@
         <v>2026-05-28</v>
       </c>
       <c r="C4" t="str">
-        <v>[EXP] 인건비 부대비용</v>
+        <v>[EXP] 4대보험 및 제세공과금</v>
       </c>
       <c r="D4" t="str">
         <v>Staff Overhead</v>
@@ -559,7 +559,7 @@
         <v>2026-05-28</v>
       </c>
       <c r="C5" t="str">
-        <v>[RENT] 공간 임차료 청구</v>
+        <v>[RENT] 사무실 임차료 청구</v>
       </c>
       <c r="D5" t="str">
         <v>Bldg</v>
@@ -591,121 +591,45 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>RENT-PAY-2026-5</v>
+        <v>MKT-AP-2026-5</v>
       </c>
       <c r="B6" t="str">
         <v>2026-05-28</v>
       </c>
       <c r="C6" t="str">
-        <v>[SETTLE] 임차료 결제 (90%)</v>
+        <v>[MKT] 마케팅 광고 집행비 인식</v>
       </c>
       <c r="D6" t="str">
-        <v>Bldg</v>
+        <v>Ad Partners</v>
       </c>
       <c r="E6" t="str">
+        <v>광고선전비</v>
+      </c>
+      <c r="F6" t="str">
+        <v>acc_826</v>
+      </c>
+      <c r="G6" t="str">
         <v>미지급금</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>acc_253</v>
       </c>
-      <c r="G6" t="str">
-        <v>보통예금</v>
-      </c>
-      <c r="H6" t="str">
-        <v>acc_103</v>
-      </c>
       <c r="I6">
-        <v>4950000</v>
+        <v>4000000</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>400000</v>
       </c>
       <c r="K6" t="str">
         <v>Expense</v>
       </c>
       <c r="L6" t="str">
-        <v>Approved</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>MKT-AP-2026-5</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-05-28</v>
-      </c>
-      <c r="C7" t="str">
-        <v>[MKT] 마케팅비 청구</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Google/FB</v>
-      </c>
-      <c r="E7" t="str">
-        <v>광고선전비</v>
-      </c>
-      <c r="F7" t="str">
-        <v>acc_826</v>
-      </c>
-      <c r="G7" t="str">
-        <v>미지급금</v>
-      </c>
-      <c r="H7" t="str">
-        <v>acc_253</v>
-      </c>
-      <c r="I7">
-        <v>4000000</v>
-      </c>
-      <c r="J7">
-        <v>400000</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Approved</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>MKT-PAY-2026-5</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2026-05-28</v>
-      </c>
-      <c r="C8" t="str">
-        <v>[SETTLE] 마케팅비 결제 (80% 우선집행)</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Google/FB</v>
-      </c>
-      <c r="E8" t="str">
-        <v>미지급금</v>
-      </c>
-      <c r="F8" t="str">
-        <v>acc_253</v>
-      </c>
-      <c r="G8" t="str">
-        <v>보통예금</v>
-      </c>
-      <c r="H8" t="str">
-        <v>acc_103</v>
-      </c>
-      <c r="I8">
-        <v>3520000</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="L8" t="str">
         <v>Approved</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>